<commit_message>
Arquivos gerados nas cores da marca (azul #1077BB e turquesa #1B9CB1); resumo mensal com logo, rodapé e PDF corrigido
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JWYj8GP4C4kzdNAx9tESJd
</commit_message>
<xml_diff>
--- a/docs/modelos/Relatorio_anterior_padrao.xlsx
+++ b/docs/modelos/Relatorio_anterior_padrao.xlsx
@@ -35,7 +35,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -45,6 +45,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="000F5F6C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1077BB"/>
       </patternFill>
     </fill>
   </fills>
@@ -60,11 +65,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -442,32 +448,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Unidade</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Titular</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>CPF</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Descrição</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Competência</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Vencimento</t>
         </is>
@@ -4549,9 +4555,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -4566,9 +4570,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -4611,9 +4613,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>

</xml_diff>